<commit_message>
Update - Wiki plant articles, first batch
Transefered plant concept files for all PvZ 1 plants from Lawnmaggedon and ZPG
</commit_message>
<xml_diff>
--- a/plant_port_checklist.xlsx
+++ b/plant_port_checklist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\rogue_garden\ideas_ressources_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11E2328-07F8-4A99-BF26-2DC94715B3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4B80963-27F1-4207-A1E7-FB5C39A15660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PvZ 1" sheetId="1" r:id="rId1"/>
@@ -2931,12 +2931,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -2960,7 +2966,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2996,6 +3002,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3335,7 +3347,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -3352,7 +3364,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -3369,7 +3381,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="11" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="6" t="s">
@@ -3386,7 +3398,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="12" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -3403,7 +3415,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="11" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -3420,7 +3432,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="11" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -3437,7 +3449,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -3454,7 +3466,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="11" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -3488,7 +3500,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -3505,7 +3517,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="11" t="s">
         <v>39</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -3522,7 +3534,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="11" t="s">
         <v>33</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -3539,7 +3551,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="11" t="s">
         <v>38</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -3556,7 +3568,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="11" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -3573,7 +3585,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="11" t="s">
         <v>36</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -3590,7 +3602,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="11" t="s">
         <v>37</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -3991,14 +4003,14 @@
         <v>1</v>
       </c>
       <c r="E40" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="7" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="11" t="s">
         <v>16</v>
       </c>
       <c r="B41" s="6" t="s">
@@ -4032,7 +4044,7 @@
       </c>
     </row>
     <row r="43" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="11" t="s">
         <v>18</v>
       </c>
       <c r="B43" s="6" t="s">
@@ -4059,14 +4071,14 @@
         <v>1</v>
       </c>
       <c r="E44" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G44" s="7" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="11" t="s">
         <v>14</v>
       </c>
       <c r="B45" s="6" t="s">
@@ -6863,7 +6875,7 @@
         <v>1</v>
       </c>
       <c r="G44" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update - Wiki plant articles, Batch 2
Cardboard plants from I, Zombie for the Training Grounds
</commit_message>
<xml_diff>
--- a/plant_port_checklist.xlsx
+++ b/plant_port_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4B80963-27F1-4207-A1E7-FB5C39A15660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69AD15FB-D231-42DF-9313-A842E545EF4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PvZ 1" sheetId="1" r:id="rId1"/>
@@ -3619,7 +3619,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="11" t="s">
         <v>84</v>
       </c>
       <c r="B18" s="6" t="s">
@@ -3636,7 +3636,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="11" t="s">
         <v>70</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -3653,7 +3653,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="11" t="s">
         <v>73</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -3670,7 +3670,7 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="11" t="s">
         <v>85</v>
       </c>
       <c r="B21" s="6" t="s">
@@ -3687,7 +3687,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="11" t="s">
         <v>82</v>
       </c>
       <c r="B22" s="6" t="s">
@@ -3704,7 +3704,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="11" t="s">
         <v>81</v>
       </c>
       <c r="B23" s="6" t="s">
@@ -3721,7 +3721,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="11" t="s">
         <v>65</v>
       </c>
       <c r="B24" s="6" t="s">
@@ -3738,7 +3738,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="11" t="s">
         <v>68</v>
       </c>
       <c r="B25" s="6" t="s">
@@ -3755,7 +3755,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="11" t="s">
         <v>72</v>
       </c>
       <c r="B26" s="6" t="s">
@@ -3772,7 +3772,7 @@
       </c>
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="11" t="s">
         <v>69</v>
       </c>
       <c r="B27" s="6" t="s">
@@ -3789,7 +3789,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="11" t="s">
         <v>74</v>
       </c>
       <c r="B28" s="6" t="s">
@@ -3806,7 +3806,7 @@
       </c>
     </row>
     <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="11" t="s">
         <v>71</v>
       </c>
       <c r="B29" s="6" t="s">
@@ -3823,7 +3823,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="11" t="s">
         <v>77</v>
       </c>
       <c r="B30" s="6" t="s">
@@ -3840,7 +3840,7 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="11" t="s">
         <v>79</v>
       </c>
       <c r="B31" s="6" t="s">
@@ -3857,7 +3857,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="11" t="s">
         <v>75</v>
       </c>
       <c r="B32" s="6" t="s">
@@ -3874,7 +3874,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="11" t="s">
         <v>80</v>
       </c>
       <c r="B33" s="6" t="s">
@@ -3891,7 +3891,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="11" t="s">
         <v>66</v>
       </c>
       <c r="B34" s="6" t="s">
@@ -3908,7 +3908,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="11" t="s">
         <v>86</v>
       </c>
       <c r="B35" s="6" t="s">
@@ -3925,7 +3925,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="11" t="s">
         <v>76</v>
       </c>
       <c r="B36" s="6" t="s">
@@ -3942,7 +3942,7 @@
       </c>
     </row>
     <row r="37" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="11" t="s">
         <v>78</v>
       </c>
       <c r="B37" s="6" t="s">
@@ -3959,7 +3959,7 @@
       </c>
     </row>
     <row r="38" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="11" t="s">
         <v>83</v>
       </c>
       <c r="B38" s="6" t="s">
@@ -3976,7 +3976,7 @@
       </c>
     </row>
     <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="11" t="s">
         <v>67</v>
       </c>
       <c r="B39" s="6" t="s">
@@ -4095,7 +4095,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="11" t="s">
         <v>19</v>
       </c>
       <c r="B46" s="6" t="s">
@@ -4112,7 +4112,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="5" t="s">
+      <c r="A47" s="11" t="s">
         <v>15</v>
       </c>
       <c r="B47" s="6" t="s">
@@ -4146,7 +4146,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="5" t="s">
+      <c r="A49" s="11" t="s">
         <v>58</v>
       </c>
       <c r="B49" s="6" t="s">
@@ -4163,7 +4163,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="5" t="s">
+      <c r="A50" s="11" t="s">
         <v>62</v>
       </c>
       <c r="B50" s="6" t="s">
@@ -4197,7 +4197,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="5" t="s">
+      <c r="A52" s="11" t="s">
         <v>27</v>
       </c>
       <c r="B52" s="6" t="s">
@@ -4214,7 +4214,7 @@
       </c>
     </row>
     <row r="53" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="5" t="s">
+      <c r="A53" s="11" t="s">
         <v>23</v>
       </c>
       <c r="B53" s="6" t="s">
@@ -4231,7 +4231,7 @@
       </c>
     </row>
     <row r="54" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="5" t="s">
+      <c r="A54" s="11" t="s">
         <v>28</v>
       </c>
       <c r="B54" s="6" t="s">
@@ -4248,7 +4248,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
+      <c r="A55" s="11" t="s">
         <v>24</v>
       </c>
       <c r="B55" s="6" t="s">
@@ -4265,7 +4265,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="5" t="s">
+      <c r="A56" s="11" t="s">
         <v>30</v>
       </c>
       <c r="B56" s="6" t="s">
@@ -4282,7 +4282,7 @@
       </c>
     </row>
     <row r="57" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="5" t="s">
+      <c r="A57" s="11" t="s">
         <v>26</v>
       </c>
       <c r="B57" s="6" t="s">
@@ -4299,7 +4299,7 @@
       </c>
     </row>
     <row r="58" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="5" t="s">
+      <c r="A58" s="11" t="s">
         <v>25</v>
       </c>
       <c r="B58" s="6" t="s">
@@ -4316,7 +4316,7 @@
       </c>
     </row>
     <row r="59" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="11" t="s">
         <v>29</v>
       </c>
       <c r="B59" s="6" t="s">
@@ -4333,7 +4333,7 @@
       </c>
     </row>
     <row r="60" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="5" t="s">
+      <c r="A60" s="11" t="s">
         <v>41</v>
       </c>
       <c r="B60" s="6" t="s">
@@ -4360,14 +4360,14 @@
         <v>1</v>
       </c>
       <c r="E61" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G61" s="7" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="5" t="s">
+      <c r="A62" s="11" t="s">
         <v>42</v>
       </c>
       <c r="B62" s="6" t="s">
@@ -4380,11 +4380,11 @@
         <v>1</v>
       </c>
       <c r="G62" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="5" t="s">
+      <c r="A63" s="11" t="s">
         <v>45</v>
       </c>
       <c r="B63" s="6" t="s">
@@ -4401,7 +4401,7 @@
       </c>
     </row>
     <row r="64" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="5" t="s">
+      <c r="A64" s="11" t="s">
         <v>43</v>
       </c>
       <c r="B64" s="6" t="s">
@@ -4418,7 +4418,7 @@
       </c>
     </row>
     <row r="65" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="11" t="s">
         <v>47</v>
       </c>
       <c r="B65" s="6" t="s">
@@ -4435,7 +4435,7 @@
       </c>
     </row>
     <row r="66" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="5" t="s">
+      <c r="A66" s="11" t="s">
         <v>48</v>
       </c>
       <c r="B66" s="6" t="s">
@@ -4452,7 +4452,7 @@
       </c>
     </row>
     <row r="67" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="5" t="s">
+      <c r="A67" s="11" t="s">
         <v>46</v>
       </c>
       <c r="B67" s="6" t="s">
@@ -4469,7 +4469,7 @@
       </c>
     </row>
     <row r="68" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="5" t="s">
+      <c r="A68" s="11" t="s">
         <v>53</v>
       </c>
       <c r="B68" s="6" t="s">
@@ -4486,7 +4486,7 @@
       </c>
     </row>
     <row r="69" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="5" t="s">
+      <c r="A69" s="11" t="s">
         <v>57</v>
       </c>
       <c r="B69" s="6" t="s">
@@ -4503,7 +4503,7 @@
       </c>
     </row>
     <row r="70" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="5" t="s">
+      <c r="A70" s="11" t="s">
         <v>50</v>
       </c>
       <c r="B70" s="6" t="s">
@@ -4520,7 +4520,7 @@
       </c>
     </row>
     <row r="71" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="5" t="s">
+      <c r="A71" s="11" t="s">
         <v>52</v>
       </c>
       <c r="B71" s="6" t="s">
@@ -4537,7 +4537,7 @@
       </c>
     </row>
     <row r="72" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="5" t="s">
+      <c r="A72" s="11" t="s">
         <v>55</v>
       </c>
       <c r="B72" s="6" t="s">
@@ -4557,7 +4557,7 @@
       </c>
     </row>
     <row r="73" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="5" t="s">
+      <c r="A73" s="11" t="s">
         <v>56</v>
       </c>
       <c r="B73" s="6" t="s">
@@ -4574,7 +4574,7 @@
       </c>
     </row>
     <row r="74" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="5" t="s">
+      <c r="A74" s="11" t="s">
         <v>51</v>
       </c>
       <c r="B74" s="6" t="s">
@@ -4591,7 +4591,7 @@
       </c>
     </row>
     <row r="75" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="5" t="s">
+      <c r="A75" s="11" t="s">
         <v>54</v>
       </c>
       <c r="B75" s="6" t="s">

</xml_diff>

<commit_message>
Update - Wiki plant articles, Batch 3
PvZ 1C and Adventures plants
</commit_message>
<xml_diff>
--- a/plant_port_checklist.xlsx
+++ b/plant_port_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69AD15FB-D231-42DF-9313-A842E545EF4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF266DD-E474-4C54-8C75-EA57F07FE2F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2966,7 +2966,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3008,6 +3008,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3472,7 +3480,7 @@
       <c r="B9" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="7" t="b">
+      <c r="C9" s="13" t="b">
         <v>1</v>
       </c>
       <c r="E9" s="7" t="b">

</xml_diff>

<commit_message>
Update - Wiki plant articles, Batch 4
PvZ 2 Lost City plants
</commit_message>
<xml_diff>
--- a/plant_port_checklist.xlsx
+++ b/plant_port_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97D13B70-F26C-4909-B557-B1CCFF1054E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6650EC9B-4EB1-4F59-B775-A6EBD8E2D1DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1817" uniqueCount="957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1819" uniqueCount="958">
   <si>
     <t>Origin Name</t>
   </si>
@@ -2905,6 +2905,9 @@
   </si>
   <si>
     <t>Frost-shroom</t>
+  </si>
+  <si>
+    <t>Sunflower Seeds</t>
   </si>
 </sst>
 </file>
@@ -2969,7 +2972,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3019,12 +3022,6 @@
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6454,7 +6451,7 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="11" t="s">
         <v>138</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -6749,7 +6746,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="11" t="s">
         <v>141</v>
       </c>
       <c r="B36" s="6" t="s">
@@ -6766,7 +6763,7 @@
       </c>
     </row>
     <row r="37" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="11" t="s">
         <v>142</v>
       </c>
       <c r="B37" s="6" t="s">
@@ -6783,7 +6780,7 @@
       </c>
     </row>
     <row r="38" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="11" t="s">
         <v>144</v>
       </c>
       <c r="B38" s="6" t="s">
@@ -6800,7 +6797,7 @@
       </c>
     </row>
     <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="11" t="s">
         <v>140</v>
       </c>
       <c r="B39" s="6" t="s">
@@ -6817,7 +6814,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="11" t="s">
         <v>143</v>
       </c>
       <c r="B40" s="6" t="s">
@@ -7948,7 +7945,7 @@
       </c>
     </row>
     <row r="106" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="14" t="s">
+      <c r="A106" s="5" t="s">
         <v>279</v>
       </c>
       <c r="B106" s="6" t="s">
@@ -11588,7 +11585,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC464112-9E41-4E5C-8F95-91067E9A4651}">
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.77734375" style="5" customWidth="1"/>
@@ -11647,13 +11644,13 @@
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>769</v>
+        <v>316</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>946</v>
+        <v>890</v>
       </c>
       <c r="C3" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="7" t="b">
         <v>0</v>
@@ -11664,10 +11661,10 @@
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>846</v>
+        <v>556</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>841</v>
+        <v>890</v>
       </c>
       <c r="C4" s="7" t="b">
         <v>0</v>
@@ -11681,13 +11678,13 @@
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>834</v>
+        <v>769</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>823</v>
+        <v>946</v>
       </c>
       <c r="C5" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="7" t="b">
         <v>0</v>
@@ -11698,7 +11695,7 @@
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>841</v>
@@ -11715,10 +11712,10 @@
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>819</v>
+        <v>834</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>820</v>
+        <v>823</v>
       </c>
       <c r="C7" s="7" t="b">
         <v>0</v>
@@ -11732,10 +11729,10 @@
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>833</v>
+        <v>848</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>823</v>
+        <v>841</v>
       </c>
       <c r="C8" s="7" t="b">
         <v>0</v>
@@ -11749,13 +11746,13 @@
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>778</v>
+        <v>819</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>782</v>
+        <v>820</v>
       </c>
       <c r="C9" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="7" t="b">
         <v>0</v>
@@ -11766,7 +11763,7 @@
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>877</v>
+        <v>833</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>823</v>
@@ -11783,13 +11780,13 @@
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>844</v>
+        <v>778</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>841</v>
+        <v>782</v>
       </c>
       <c r="C11" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="7" t="b">
         <v>0</v>
@@ -11800,7 +11797,7 @@
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>829</v>
+        <v>877</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>823</v>
@@ -11817,27 +11814,27 @@
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>775</v>
+        <v>844</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>776</v>
+        <v>841</v>
       </c>
       <c r="C13" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>845</v>
+        <v>936</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>841</v>
+        <v>890</v>
       </c>
       <c r="C14" s="7" t="b">
         <v>0</v>
@@ -11851,7 +11848,7 @@
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>823</v>
@@ -11868,16 +11865,16 @@
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>836</v>
+        <v>886</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>823</v>
+        <v>890</v>
       </c>
       <c r="C16" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E16" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="7" t="b">
         <v>0</v>
@@ -11885,27 +11882,27 @@
     </row>
     <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>880</v>
+        <v>775</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>841</v>
+        <v>776</v>
       </c>
       <c r="C17" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>822</v>
+        <v>845</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>823</v>
+        <v>841</v>
       </c>
       <c r="C18" s="7" t="b">
         <v>0</v>
@@ -11919,10 +11916,10 @@
     </row>
     <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>785</v>
+        <v>831</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>788</v>
+        <v>823</v>
       </c>
       <c r="C19" s="7" t="b">
         <v>0</v>
@@ -11936,10 +11933,10 @@
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>879</v>
+        <v>836</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>841</v>
+        <v>823</v>
       </c>
       <c r="C20" s="7" t="b">
         <v>0</v>
@@ -11953,10 +11950,10 @@
     </row>
     <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>789</v>
+        <v>882</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>791</v>
+        <v>890</v>
       </c>
       <c r="C21" s="7" t="b">
         <v>0</v>
@@ -11970,13 +11967,13 @@
     </row>
     <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>786</v>
+        <v>880</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>788</v>
+        <v>841</v>
       </c>
       <c r="C22" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="7" t="b">
         <v>0</v>
@@ -11987,10 +11984,10 @@
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>847</v>
+        <v>822</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>841</v>
+        <v>823</v>
       </c>
       <c r="C23" s="7" t="b">
         <v>0</v>
@@ -12004,10 +12001,10 @@
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>830</v>
+        <v>785</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>823</v>
+        <v>788</v>
       </c>
       <c r="C24" s="7" t="b">
         <v>0</v>
@@ -12021,10 +12018,10 @@
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>875</v>
+        <v>914</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>823</v>
+        <v>908</v>
       </c>
       <c r="C25" s="7" t="b">
         <v>0</v>
@@ -12038,10 +12035,10 @@
     </row>
     <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>798</v>
+        <v>933</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>793</v>
+        <v>908</v>
       </c>
       <c r="C26" s="7" t="b">
         <v>0</v>
@@ -12055,10 +12052,10 @@
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>796</v>
+        <v>910</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>793</v>
+        <v>908</v>
       </c>
       <c r="C27" s="7" t="b">
         <v>0</v>
@@ -12072,10 +12069,10 @@
     </row>
     <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>795</v>
+        <v>912</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>793</v>
+        <v>908</v>
       </c>
       <c r="C28" s="7" t="b">
         <v>0</v>
@@ -12089,10 +12086,10 @@
     </row>
     <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>794</v>
+        <v>911</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>793</v>
+        <v>908</v>
       </c>
       <c r="C29" s="7" t="b">
         <v>0</v>
@@ -12106,10 +12103,10 @@
     </row>
     <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>797</v>
+        <v>909</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>793</v>
+        <v>908</v>
       </c>
       <c r="C30" s="7" t="b">
         <v>0</v>
@@ -12123,16 +12120,19 @@
     </row>
     <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>784</v>
+        <v>913</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>788</v>
+        <v>908</v>
       </c>
       <c r="C31" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E31" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>938</v>
       </c>
       <c r="G31" s="7" t="b">
         <v>0</v>
@@ -12140,10 +12140,10 @@
     </row>
     <row r="32" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>826</v>
+        <v>922</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>823</v>
+        <v>908</v>
       </c>
       <c r="C32" s="7" t="b">
         <v>0</v>
@@ -12157,10 +12157,10 @@
     </row>
     <row r="33" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>790</v>
+        <v>879</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>791</v>
+        <v>841</v>
       </c>
       <c r="C33" s="7" t="b">
         <v>0</v>
@@ -12174,10 +12174,10 @@
     </row>
     <row r="34" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="C34" s="7" t="b">
         <v>0</v>
@@ -12191,16 +12191,16 @@
     </row>
     <row r="35" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>874</v>
+        <v>924</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>820</v>
+        <v>890</v>
       </c>
       <c r="C35" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E35" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" s="7" t="b">
         <v>0</v>
@@ -12208,16 +12208,16 @@
     </row>
     <row r="36" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>770</v>
+        <v>786</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>771</v>
+        <v>788</v>
       </c>
       <c r="C36" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" s="7" t="b">
         <v>0</v>
@@ -12225,10 +12225,10 @@
     </row>
     <row r="37" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>849</v>
+        <v>907</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>841</v>
+        <v>899</v>
       </c>
       <c r="C37" s="7" t="b">
         <v>0</v>
@@ -12242,7 +12242,7 @@
     </row>
     <row r="38" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>841</v>
@@ -12259,10 +12259,10 @@
     </row>
     <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>878</v>
+        <v>935</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>841</v>
+        <v>916</v>
       </c>
       <c r="C39" s="7" t="b">
         <v>0</v>
@@ -12276,16 +12276,16 @@
     </row>
     <row r="40" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>837</v>
+        <v>896</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>823</v>
+        <v>900</v>
       </c>
       <c r="C40" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E40" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="7" t="b">
         <v>0</v>
@@ -12293,10 +12293,10 @@
     </row>
     <row r="41" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>853</v>
+        <v>884</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>841</v>
+        <v>890</v>
       </c>
       <c r="C41" s="7" t="b">
         <v>0</v>
@@ -12310,7 +12310,7 @@
     </row>
     <row r="42" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>838</v>
+        <v>830</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>823</v>
@@ -12327,10 +12327,10 @@
     </row>
     <row r="43" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>781</v>
+        <v>875</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>782</v>
+        <v>823</v>
       </c>
       <c r="C43" s="7" t="b">
         <v>0</v>
@@ -12344,10 +12344,10 @@
     </row>
     <row r="44" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>876</v>
+        <v>798</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>823</v>
+        <v>793</v>
       </c>
       <c r="C44" s="7" t="b">
         <v>0</v>
@@ -12361,16 +12361,16 @@
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>947</v>
+        <v>796</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>841</v>
+        <v>793</v>
       </c>
       <c r="C45" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E45" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45" s="7" t="b">
         <v>0</v>
@@ -12378,10 +12378,10 @@
     </row>
     <row r="46" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>774</v>
+        <v>795</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>776</v>
+        <v>793</v>
       </c>
       <c r="C46" s="7" t="b">
         <v>0</v>
@@ -12395,10 +12395,10 @@
     </row>
     <row r="47" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>779</v>
+        <v>794</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>782</v>
+        <v>793</v>
       </c>
       <c r="C47" s="7" t="b">
         <v>0</v>
@@ -12412,10 +12412,10 @@
     </row>
     <row r="48" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>780</v>
+        <v>797</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>782</v>
+        <v>793</v>
       </c>
       <c r="C48" s="7" t="b">
         <v>0</v>
@@ -12429,10 +12429,10 @@
     </row>
     <row r="49" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>777</v>
+        <v>920</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>782</v>
+        <v>921</v>
       </c>
       <c r="C49" s="7" t="b">
         <v>0</v>
@@ -12446,10 +12446,10 @@
     </row>
     <row r="50" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>772</v>
+        <v>784</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>773</v>
+        <v>788</v>
       </c>
       <c r="C50" s="7" t="b">
         <v>0</v>
@@ -12463,10 +12463,10 @@
     </row>
     <row r="51" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>824</v>
+        <v>918</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>823</v>
+        <v>916</v>
       </c>
       <c r="C51" s="7" t="b">
         <v>0</v>
@@ -12480,10 +12480,10 @@
     </row>
     <row r="52" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>855</v>
+        <v>917</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>841</v>
+        <v>916</v>
       </c>
       <c r="C52" s="7" t="b">
         <v>0</v>
@@ -12497,10 +12497,10 @@
     </row>
     <row r="53" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>854</v>
+        <v>937</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>841</v>
+        <v>916</v>
       </c>
       <c r="C53" s="7" t="b">
         <v>0</v>
@@ -12514,10 +12514,10 @@
     </row>
     <row r="54" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>828</v>
+        <v>919</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>823</v>
+        <v>916</v>
       </c>
       <c r="C54" s="7" t="b">
         <v>0</v>
@@ -12531,7 +12531,7 @@
     </row>
     <row r="55" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>839</v>
+        <v>826</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>823</v>
@@ -12540,10 +12540,7 @@
         <v>0</v>
       </c>
       <c r="E55" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F55" s="5" t="s">
-        <v>868</v>
+        <v>0</v>
       </c>
       <c r="G55" s="7" t="b">
         <v>0</v>
@@ -12551,10 +12548,10 @@
     </row>
     <row r="56" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>60</v>
+        <v>791</v>
       </c>
       <c r="C56" s="7" t="b">
         <v>0</v>
@@ -12568,10 +12565,10 @@
     </row>
     <row r="57" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
-        <v>842</v>
+        <v>787</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>841</v>
+        <v>788</v>
       </c>
       <c r="C57" s="7" t="b">
         <v>0</v>
@@ -12585,10 +12582,10 @@
     </row>
     <row r="58" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
-        <v>840</v>
+        <v>874</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="C58" s="7" t="b">
         <v>0</v>
@@ -12602,10 +12599,10 @@
     </row>
     <row r="59" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>832</v>
+        <v>887</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>823</v>
+        <v>890</v>
       </c>
       <c r="C59" s="7" t="b">
         <v>0</v>
@@ -12619,16 +12616,16 @@
     </row>
     <row r="60" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>852</v>
+        <v>770</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>841</v>
+        <v>771</v>
       </c>
       <c r="C60" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E60" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G60" s="7" t="b">
         <v>0</v>
@@ -12636,10 +12633,10 @@
     </row>
     <row r="61" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
-        <v>856</v>
+        <v>889</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>841</v>
+        <v>890</v>
       </c>
       <c r="C61" s="7" t="b">
         <v>0</v>
@@ -12653,7 +12650,7 @@
     </row>
     <row r="62" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>841</v>
@@ -12670,10 +12667,10 @@
     </row>
     <row r="63" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>835</v>
+        <v>843</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>823</v>
+        <v>841</v>
       </c>
       <c r="C63" s="7" t="b">
         <v>0</v>
@@ -12687,10 +12684,10 @@
     </row>
     <row r="64" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
-        <v>825</v>
+        <v>929</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>823</v>
+        <v>908</v>
       </c>
       <c r="C64" s="7" t="b">
         <v>0</v>
@@ -12704,10 +12701,10 @@
     </row>
     <row r="65" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
-        <v>827</v>
+        <v>928</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>823</v>
+        <v>899</v>
       </c>
       <c r="C65" s="7" t="b">
         <v>0</v>
@@ -12721,10 +12718,10 @@
     </row>
     <row r="66" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
-        <v>821</v>
+        <v>930</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>820</v>
+        <v>916</v>
       </c>
       <c r="C66" s="7" t="b">
         <v>0</v>
@@ -12738,7 +12735,7 @@
     </row>
     <row r="67" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
-        <v>850</v>
+        <v>878</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>841</v>
@@ -12755,10 +12752,10 @@
     </row>
     <row r="68" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
-        <v>556</v>
+        <v>931</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>890</v>
+        <v>900</v>
       </c>
       <c r="C68" s="7" t="b">
         <v>0</v>
@@ -12772,7 +12769,7 @@
     </row>
     <row r="69" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B69" s="6" t="s">
         <v>890</v>
@@ -12781,7 +12778,7 @@
         <v>0</v>
       </c>
       <c r="E69" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G69" s="7" t="b">
         <v>0</v>
@@ -12789,10 +12786,10 @@
     </row>
     <row r="70" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
-        <v>882</v>
+        <v>903</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>890</v>
+        <v>899</v>
       </c>
       <c r="C70" s="7" t="b">
         <v>0</v>
@@ -12806,10 +12803,10 @@
     </row>
     <row r="71" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
-        <v>914</v>
+        <v>905</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="C71" s="7" t="b">
         <v>0</v>
@@ -12823,10 +12820,10 @@
     </row>
     <row r="72" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
-        <v>910</v>
+        <v>902</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="C72" s="7" t="b">
         <v>0</v>
@@ -12840,10 +12837,10 @@
     </row>
     <row r="73" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
-        <v>912</v>
+        <v>904</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="C73" s="7" t="b">
         <v>0</v>
@@ -12857,10 +12854,10 @@
     </row>
     <row r="74" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
-        <v>911</v>
+        <v>901</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="C74" s="7" t="b">
         <v>0</v>
@@ -12874,10 +12871,10 @@
     </row>
     <row r="75" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>909</v>
+        <v>923</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="C75" s="7" t="b">
         <v>0</v>
@@ -12891,19 +12888,16 @@
     </row>
     <row r="76" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
-        <v>913</v>
+        <v>837</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>908</v>
+        <v>823</v>
       </c>
       <c r="C76" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E76" s="7" t="b">
         <v>1</v>
-      </c>
-      <c r="F76" s="5" t="s">
-        <v>938</v>
       </c>
       <c r="G76" s="7" t="b">
         <v>0</v>
@@ -12911,10 +12905,10 @@
     </row>
     <row r="77" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>922</v>
+        <v>853</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>908</v>
+        <v>841</v>
       </c>
       <c r="C77" s="7" t="b">
         <v>0</v>
@@ -12928,16 +12922,16 @@
     </row>
     <row r="78" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
-        <v>924</v>
+        <v>838</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>890</v>
+        <v>823</v>
       </c>
       <c r="C78" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E78" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G78" s="7" t="b">
         <v>0</v>
@@ -12945,10 +12939,10 @@
     </row>
     <row r="79" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
-        <v>907</v>
+        <v>781</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>899</v>
+        <v>782</v>
       </c>
       <c r="C79" s="7" t="b">
         <v>0</v>
@@ -12962,10 +12956,10 @@
     </row>
     <row r="80" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
-        <v>896</v>
+        <v>876</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>900</v>
+        <v>823</v>
       </c>
       <c r="C80" s="7" t="b">
         <v>0</v>
@@ -12979,7 +12973,7 @@
     </row>
     <row r="81" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B81" s="6" t="s">
         <v>890</v>
@@ -12996,16 +12990,16 @@
     </row>
     <row r="82" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
-        <v>920</v>
+        <v>947</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>921</v>
+        <v>841</v>
       </c>
       <c r="C82" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E82" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G82" s="7" t="b">
         <v>0</v>
@@ -13013,10 +13007,10 @@
     </row>
     <row r="83" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
-        <v>918</v>
+        <v>774</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>916</v>
+        <v>776</v>
       </c>
       <c r="C83" s="7" t="b">
         <v>0</v>
@@ -13030,10 +13024,10 @@
     </row>
     <row r="84" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
-        <v>917</v>
+        <v>906</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>916</v>
+        <v>899</v>
       </c>
       <c r="C84" s="7" t="b">
         <v>0</v>
@@ -13047,10 +13041,10 @@
     </row>
     <row r="85" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
-        <v>919</v>
+        <v>779</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>916</v>
+        <v>782</v>
       </c>
       <c r="C85" s="7" t="b">
         <v>0</v>
@@ -13064,10 +13058,10 @@
     </row>
     <row r="86" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
-        <v>887</v>
+        <v>780</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>890</v>
+        <v>782</v>
       </c>
       <c r="C86" s="7" t="b">
         <v>0</v>
@@ -13081,10 +13075,10 @@
     </row>
     <row r="87" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
-        <v>889</v>
+        <v>777</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>890</v>
+        <v>782</v>
       </c>
       <c r="C87" s="7" t="b">
         <v>0</v>
@@ -13098,10 +13092,10 @@
     </row>
     <row r="88" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
-        <v>885</v>
+        <v>772</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>890</v>
+        <v>773</v>
       </c>
       <c r="C88" s="7" t="b">
         <v>0</v>
@@ -13115,10 +13109,10 @@
     </row>
     <row r="89" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
-        <v>903</v>
+        <v>824</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>899</v>
+        <v>823</v>
       </c>
       <c r="C89" s="7" t="b">
         <v>0</v>
@@ -13132,10 +13126,10 @@
     </row>
     <row r="90" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
-        <v>905</v>
+        <v>855</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>899</v>
+        <v>841</v>
       </c>
       <c r="C90" s="7" t="b">
         <v>0</v>
@@ -13149,10 +13143,10 @@
     </row>
     <row r="91" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
-        <v>902</v>
+        <v>854</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>899</v>
+        <v>841</v>
       </c>
       <c r="C91" s="7" t="b">
         <v>0</v>
@@ -13166,10 +13160,10 @@
     </row>
     <row r="92" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
-        <v>904</v>
+        <v>828</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>899</v>
+        <v>823</v>
       </c>
       <c r="C92" s="7" t="b">
         <v>0</v>
@@ -13183,16 +13177,19 @@
     </row>
     <row r="93" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
-        <v>901</v>
+        <v>839</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>899</v>
+        <v>823</v>
       </c>
       <c r="C93" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E93" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F93" s="5" t="s">
+        <v>868</v>
       </c>
       <c r="G93" s="7" t="b">
         <v>0</v>
@@ -13200,10 +13197,10 @@
     </row>
     <row r="94" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
-        <v>923</v>
+        <v>792</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>899</v>
+        <v>60</v>
       </c>
       <c r="C94" s="7" t="b">
         <v>0</v>
@@ -13217,10 +13214,10 @@
     </row>
     <row r="95" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
-        <v>883</v>
+        <v>842</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>890</v>
+        <v>841</v>
       </c>
       <c r="C95" s="7" t="b">
         <v>0</v>
@@ -13234,10 +13231,10 @@
     </row>
     <row r="96" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
-        <v>906</v>
+        <v>957</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>899</v>
+        <v>823</v>
       </c>
       <c r="C96" s="7" t="b">
         <v>0</v>
@@ -13251,19 +13248,16 @@
     </row>
     <row r="97" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
-        <v>915</v>
+        <v>840</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>908</v>
+        <v>823</v>
       </c>
       <c r="C97" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E97" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F97" s="5" t="s">
-        <v>926</v>
+        <v>0</v>
       </c>
       <c r="G97" s="7" t="b">
         <v>0</v>
@@ -13271,19 +13265,16 @@
     </row>
     <row r="98" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
-        <v>895</v>
+        <v>832</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>900</v>
+        <v>823</v>
       </c>
       <c r="C98" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E98" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F98" s="5" t="s">
-        <v>925</v>
+        <v>0</v>
       </c>
       <c r="G98" s="7" t="b">
         <v>0</v>
@@ -13291,10 +13282,10 @@
     </row>
     <row r="99" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
-        <v>897</v>
+        <v>852</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>900</v>
+        <v>841</v>
       </c>
       <c r="C99" s="7" t="b">
         <v>0</v>
@@ -13308,10 +13299,10 @@
     </row>
     <row r="100" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
-        <v>898</v>
+        <v>856</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>900</v>
+        <v>841</v>
       </c>
       <c r="C100" s="7" t="b">
         <v>0</v>
@@ -13325,10 +13316,10 @@
     </row>
     <row r="101" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
-        <v>891</v>
+        <v>932</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>900</v>
+        <v>908</v>
       </c>
       <c r="C101" s="7" t="b">
         <v>0</v>
@@ -13342,16 +13333,19 @@
     </row>
     <row r="102" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
-        <v>892</v>
+        <v>915</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>900</v>
+        <v>908</v>
       </c>
       <c r="C102" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E102" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F102" s="5" t="s">
+        <v>926</v>
       </c>
       <c r="G102" s="7" t="b">
         <v>0</v>
@@ -13359,10 +13353,10 @@
     </row>
     <row r="103" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
-        <v>893</v>
+        <v>851</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>900</v>
+        <v>841</v>
       </c>
       <c r="C103" s="7" t="b">
         <v>0</v>
@@ -13376,10 +13370,10 @@
     </row>
     <row r="104" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
-        <v>894</v>
+        <v>835</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>900</v>
+        <v>823</v>
       </c>
       <c r="C104" s="7" t="b">
         <v>0</v>
@@ -13393,16 +13387,19 @@
     </row>
     <row r="105" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
-        <v>888</v>
+        <v>895</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>890</v>
+        <v>900</v>
       </c>
       <c r="C105" s="7" t="b">
         <v>0</v>
       </c>
       <c r="E105" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F105" s="5" t="s">
+        <v>925</v>
       </c>
       <c r="G105" s="7" t="b">
         <v>0</v>
@@ -13410,7 +13407,7 @@
     </row>
     <row r="106" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
-        <v>927</v>
+        <v>897</v>
       </c>
       <c r="B106" s="6" t="s">
         <v>900</v>
@@ -13427,10 +13424,10 @@
     </row>
     <row r="107" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
-        <v>928</v>
+        <v>898</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="C107" s="7" t="b">
         <v>0</v>
@@ -13444,10 +13441,10 @@
     </row>
     <row r="108" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
-        <v>929</v>
+        <v>891</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>908</v>
+        <v>900</v>
       </c>
       <c r="C108" s="7" t="b">
         <v>0</v>
@@ -13461,10 +13458,10 @@
     </row>
     <row r="109" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
-        <v>930</v>
+        <v>892</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>916</v>
+        <v>900</v>
       </c>
       <c r="C109" s="7" t="b">
         <v>0</v>
@@ -13478,7 +13475,7 @@
     </row>
     <row r="110" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
-        <v>931</v>
+        <v>893</v>
       </c>
       <c r="B110" s="6" t="s">
         <v>900</v>
@@ -13495,10 +13492,10 @@
     </row>
     <row r="111" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
-        <v>932</v>
+        <v>927</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>908</v>
+        <v>900</v>
       </c>
       <c r="C111" s="7" t="b">
         <v>0</v>
@@ -13512,10 +13509,10 @@
     </row>
     <row r="112" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="5" t="s">
-        <v>316</v>
+        <v>894</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>890</v>
+        <v>900</v>
       </c>
       <c r="C112" s="7" t="b">
         <v>0</v>
@@ -13529,10 +13526,10 @@
     </row>
     <row r="113" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>908</v>
+        <v>890</v>
       </c>
       <c r="C113" s="7" t="b">
         <v>0</v>
@@ -13546,10 +13543,10 @@
     </row>
     <row r="114" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
-        <v>934</v>
+        <v>825</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>890</v>
+        <v>823</v>
       </c>
       <c r="C114" s="7" t="b">
         <v>0</v>
@@ -13563,10 +13560,10 @@
     </row>
     <row r="115" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
-        <v>935</v>
+        <v>827</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>916</v>
+        <v>823</v>
       </c>
       <c r="C115" s="7" t="b">
         <v>0</v>
@@ -13580,7 +13577,7 @@
     </row>
     <row r="116" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
-        <v>936</v>
+        <v>888</v>
       </c>
       <c r="B116" s="6" t="s">
         <v>890</v>
@@ -13597,10 +13594,10 @@
     </row>
     <row r="117" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
-        <v>937</v>
+        <v>821</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>916</v>
+        <v>820</v>
       </c>
       <c r="C117" s="7" t="b">
         <v>0</v>
@@ -13612,9 +13609,26 @@
         <v>0</v>
       </c>
     </row>
+    <row r="118" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="5" t="s">
+        <v>850</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>841</v>
+      </c>
+      <c r="C118" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E118" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G118" s="7" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F67">
-    <sortCondition ref="A1:A67"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G118">
+    <sortCondition ref="A1:A118"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update - Wiki plant articles, Batch 5 + Sweet Pea art
PvZ 2 worlds: Dark Ages, Jurassic Marsh, Neon Mixtape Tour,
</commit_message>
<xml_diff>
--- a/plant_port_checklist.xlsx
+++ b/plant_port_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6650EC9B-4EB1-4F59-B775-A6EBD8E2D1DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CBBB3F-3EEF-4A8D-9E8A-8D8D4B41F3CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20040" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PvZ 1" sheetId="1" r:id="rId1"/>
@@ -6264,7 +6264,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="11" t="s">
         <v>153</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -6661,7 +6661,7 @@
       </c>
     </row>
     <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="11" t="s">
         <v>162</v>
       </c>
       <c r="B31" s="6" t="s">
@@ -6678,7 +6678,7 @@
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="11" t="s">
         <v>807</v>
       </c>
       <c r="B32" s="6" t="s">
@@ -6695,7 +6695,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="11" t="s">
         <v>164</v>
       </c>
       <c r="B33" s="6" t="s">
@@ -6729,7 +6729,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="11" t="s">
         <v>161</v>
       </c>
       <c r="B35" s="6" t="s">
@@ -6916,7 +6916,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="11" t="s">
         <v>157</v>
       </c>
       <c r="B46" s="6" t="s">
@@ -6933,7 +6933,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="5" t="s">
+      <c r="A47" s="11" t="s">
         <v>160</v>
       </c>
       <c r="B47" s="6" t="s">
@@ -6950,7 +6950,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="5" t="s">
+      <c r="A48" s="11" t="s">
         <v>156</v>
       </c>
       <c r="B48" s="6" t="s">
@@ -6967,7 +6967,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="5" t="s">
+      <c r="A49" s="11" t="s">
         <v>159</v>
       </c>
       <c r="B49" s="6" t="s">
@@ -6984,7 +6984,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="5" t="s">
+      <c r="A50" s="11" t="s">
         <v>158</v>
       </c>
       <c r="B50" s="6" t="s">
@@ -7008,7 +7008,7 @@
         <v>60</v>
       </c>
       <c r="C51" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E51" s="7" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update - Wiki plant articles, Batch 6
PvZ 2 worlds Big Wave Beach and Modern Day
</commit_message>
<xml_diff>
--- a/plant_port_checklist.xlsx
+++ b/plant_port_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CBBB3F-3EEF-4A8D-9E8A-8D8D4B41F3CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F59451B-FB77-4DC9-9C06-1630FDB95C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20040" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PvZ 1" sheetId="1" r:id="rId1"/>
@@ -6213,7 +6213,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="11" t="s">
         <v>169</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -6230,7 +6230,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="11" t="s">
         <v>167</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -6247,7 +6247,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="11" t="s">
         <v>168</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -6831,7 +6831,7 @@
       </c>
     </row>
     <row r="41" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="11" t="s">
         <v>173</v>
       </c>
       <c r="B41" s="6" t="s">
@@ -6848,7 +6848,7 @@
       </c>
     </row>
     <row r="42" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="11" t="s">
         <v>174</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -6865,7 +6865,7 @@
       </c>
     </row>
     <row r="43" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="11" t="s">
         <v>170</v>
       </c>
       <c r="B43" s="6" t="s">
@@ -6882,7 +6882,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="11" t="s">
         <v>171</v>
       </c>
       <c r="B44" s="6" t="s">
@@ -6899,7 +6899,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="11" t="s">
         <v>172</v>
       </c>
       <c r="B45" s="6" t="s">

</xml_diff>

<commit_message>
Update - Wiki plant articles, Batch 7
</commit_message>
<xml_diff>
--- a/plant_port_checklist.xlsx
+++ b/plant_port_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F59451B-FB77-4DC9-9C06-1630FDB95C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5690EC00-7029-4C9E-8D20-F86642346254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20025" yWindow="-21600" windowWidth="17415" windowHeight="20985" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PvZ 1" sheetId="1" r:id="rId1"/>
@@ -4841,7 +4841,7 @@
       <c r="E14" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="11" t="s">
         <v>943</v>
       </c>
     </row>
@@ -4855,7 +4855,7 @@
       <c r="E15" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="11" t="s">
         <v>944</v>
       </c>
     </row>
@@ -4869,7 +4869,7 @@
       <c r="E16" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="11" t="s">
         <v>945</v>
       </c>
     </row>
@@ -4897,7 +4897,7 @@
       <c r="E18" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="11" t="s">
         <v>954</v>
       </c>
     </row>
@@ -6485,7 +6485,7 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="11" t="s">
         <v>200</v>
       </c>
       <c r="B21" s="6" t="s">
@@ -7395,7 +7395,7 @@
       </c>
     </row>
     <row r="74" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="5" t="s">
+      <c r="A74" s="11" t="s">
         <v>183</v>
       </c>
       <c r="B74" s="6" t="s">
@@ -7429,7 +7429,7 @@
       </c>
     </row>
     <row r="76" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="5" t="s">
+      <c r="A76" s="11" t="s">
         <v>192</v>
       </c>
       <c r="B76" s="6" t="s">
@@ -7446,7 +7446,7 @@
       </c>
     </row>
     <row r="77" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="5" t="s">
+      <c r="A77" s="11" t="s">
         <v>184</v>
       </c>
       <c r="B77" s="6" t="s">
@@ -8662,7 +8662,7 @@
       </c>
     </row>
     <row r="148" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="5" t="s">
+      <c r="A148" s="11" t="s">
         <v>230</v>
       </c>
       <c r="B148" s="6" t="s">

</xml_diff>

<commit_message>
Update - Concept Files
</commit_message>
<xml_diff>
--- a/plant_port_checklist.xlsx
+++ b/plant_port_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_rogue_garden_wiki\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193158CB-FD3F-4721-A004-BACF37073620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C989C5-A2F5-47DF-9B79-D6B195853999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="7965" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PvZ 1" sheetId="1" r:id="rId1"/>
@@ -2914,7 +2914,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2932,6 +2932,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Trebuchet MS"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1" tint="0.499984740745262"/>
       <name val="Trebuchet MS"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2972,7 +2979,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3022,6 +3029,9 @@
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3497,7 +3507,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="11" t="s">
         <v>35</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -4007,7 +4017,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="11" t="s">
         <v>21</v>
       </c>
       <c r="B40" s="6" t="s">
@@ -4041,7 +4051,7 @@
       </c>
     </row>
     <row r="42" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="11" t="s">
         <v>17</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -4075,7 +4085,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="11" t="s">
         <v>20</v>
       </c>
       <c r="B44" s="6" t="s">
@@ -4143,7 +4153,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="5" t="s">
+      <c r="A48" s="14" t="s">
         <v>61</v>
       </c>
       <c r="B48" s="6" t="s">
@@ -4194,7 +4204,7 @@
       </c>
     </row>
     <row r="51" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="14" t="s">
         <v>63</v>
       </c>
       <c r="B51" s="6" t="s">
@@ -4364,7 +4374,7 @@
       </c>
     </row>
     <row r="61" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="5" t="s">
+      <c r="A61" s="11" t="s">
         <v>44</v>
       </c>
       <c r="B61" s="6" t="s">
@@ -5546,7 +5556,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="14" t="s">
         <v>105</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -5563,7 +5573,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="14" t="s">
         <v>100</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -5580,7 +5590,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="14" t="s">
         <v>101</v>
       </c>
       <c r="B4" s="6" t="s">
@@ -5597,7 +5607,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="14" t="s">
         <v>104</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -5637,7 +5647,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="14" t="s">
         <v>89</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -5654,7 +5664,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="14" t="s">
         <v>93</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -5671,7 +5681,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="14" t="s">
         <v>94</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -5688,7 +5698,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="14" t="s">
         <v>98</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -5705,7 +5715,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="14" t="s">
         <v>91</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -5722,7 +5732,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="14" t="s">
         <v>92</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -5756,7 +5766,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="14" t="s">
         <v>102</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -5773,7 +5783,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="14" t="s">
         <v>90</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -5908,7 +5918,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="14" t="s">
         <v>115</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -5925,7 +5935,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="14" t="s">
         <v>108</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -5942,7 +5952,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="14" t="s">
         <v>119</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -5976,7 +5986,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="14" t="s">
         <v>116</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -5993,7 +6003,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="14" t="s">
         <v>120</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -6027,7 +6037,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="14" t="s">
         <v>107</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -6044,7 +6054,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="14" t="s">
         <v>118</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -6061,7 +6071,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="14" t="s">
         <v>110</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -6078,7 +6088,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="14" t="s">
         <v>121</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -6468,7 +6478,7 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="11" t="s">
         <v>204</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -6508,7 +6518,7 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="11" t="s">
         <v>196</v>
       </c>
       <c r="B22" s="6" t="s">

</xml_diff>